<commit_message>
Update link ảnh sp
</commit_message>
<xml_diff>
--- a/vnop_purchase/static/xlsx/import_san_pham.xlsx
+++ b/vnop_purchase/static/xlsx/import_san_pham.xlsx
@@ -792,7 +792,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="A3" authorId="0" shapeId="0">
+    <comment ref="A2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -801,7 +801,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="B3" authorId="0" shapeId="0">
+    <comment ref="B2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -809,7 +809,7 @@
     Mã tự đinh nghĩa nếu muốn</t>
       </text>
     </comment>
-    <comment ref="C3" authorId="0" shapeId="0">
+    <comment ref="C2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -823,7 +823,7 @@
 07 - Dịch vụ</t>
       </text>
     </comment>
-    <comment ref="D3" authorId="0" shapeId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -831,7 +831,7 @@
     Theo danh sách nhóm đã đăng ký trên phần mềm sẽ gửi bảng riêng</t>
       </text>
     </comment>
-    <comment ref="E3" authorId="0" shapeId="0">
+    <comment ref="E2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -842,7 +842,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="F3" authorId="0" shapeId="0">
+    <comment ref="F2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -850,7 +850,7 @@
     Theo mã NCC trên phần mềm đã đăng ký hoặc bỏ trống</t>
       </text>
     </comment>
-    <comment ref="G3" authorId="0" shapeId="0">
+    <comment ref="G2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -858,7 +858,7 @@
     Tên đên vị Xuất khấu</t>
       </text>
     </comment>
-    <comment ref="H3" authorId="0" shapeId="0">
+    <comment ref="H2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -867,7 +867,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="I3" authorId="0" shapeId="0">
+    <comment ref="I2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -875,7 +875,7 @@
     Tên hàng đầy đủ</t>
       </text>
     </comment>
-    <comment ref="J3" authorId="0" shapeId="0">
+    <comment ref="J2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -883,7 +883,7 @@
     Tên hàng rút gon - nếu không thì điền giống tên đầy đủ</t>
       </text>
     </comment>
-    <comment ref="K3" authorId="0" shapeId="0">
+    <comment ref="K2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -891,7 +891,7 @@
     Tên hàng để viết hoá đơn (có thể là tên chung của nhiều mã hàng)</t>
       </text>
     </comment>
-    <comment ref="L3" authorId="0" shapeId="0">
+    <comment ref="L2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -900,7 +900,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="M3" authorId="0" shapeId="0">
+    <comment ref="M2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -909,7 +909,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="N3" authorId="0" shapeId="0">
+    <comment ref="N2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -917,7 +917,7 @@
     Mặc đinh là 01 - hàng hoá đếm được</t>
       </text>
     </comment>
-    <comment ref="O3" authorId="0" shapeId="0">
+    <comment ref="O2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -926,7 +926,7 @@
 phần lớn là CAI</t>
       </text>
     </comment>
-    <comment ref="P3" authorId="0" shapeId="0">
+    <comment ref="P2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -935,7 +935,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="Q3" authorId="0" shapeId="0">
+    <comment ref="Q2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -943,7 +943,7 @@
     Giá list nếu có (chỉ đinh thị trường bán lẻ theo giá này) giá bao gồm thuế</t>
       </text>
     </comment>
-    <comment ref="T3" authorId="0" shapeId="0">
+    <comment ref="T2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -958,7 +958,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="U3" authorId="0" shapeId="0">
+    <comment ref="U2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -972,7 +972,7 @@
 D0 - hàng hoá đơn trực tiếp</t>
       </text>
     </comment>
-    <comment ref="V3" authorId="0" shapeId="0">
+    <comment ref="V2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -983,7 +983,7 @@
 3- Không thể dán tem</t>
       </text>
     </comment>
-    <comment ref="X3" authorId="0" shapeId="0">
+    <comment ref="X2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -992,7 +992,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="Y3" authorId="0" shapeId="0">
+    <comment ref="Y2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1000,75 +1000,75 @@
     Ký hiệu mầu đối với gọng</t>
       </text>
     </comment>
-    <comment ref="Z3" authorId="0" shapeId="0">
+    <comment ref="Z2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Trung Đỗ Kiên:
 Look up danh mục </t>
       </text>
     </comment>
-    <comment ref="AB3" authorId="0" shapeId="0">
+    <comment ref="AB2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Đã có -- Bổ sung thêm giá trị 3. Unisex</t>
       </text>
     </comment>
-    <comment ref="AC3" authorId="0" shapeId="0">
+    <comment ref="AC2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Thêm danh mục dáng mắt</t>
       </text>
     </comment>
-    <comment ref="AD3" authorId="0" shapeId="0">
+    <comment ref="AD2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 look up danh mục</t>
       </text>
     </comment>
-    <comment ref="AE3" authorId="0" shapeId="0">
+    <comment ref="AE2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Look up danh mục</t>
       </text>
     </comment>
-    <comment ref="AF3" authorId="0" shapeId="0">
+    <comment ref="AF2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Look up danh mục vật liệu gọng/kính
 Tách riêng danh mục vật liệu với mắt</t>
       </text>
     </comment>
-    <comment ref="AJ3" authorId="0" shapeId="0">
+    <comment ref="AJ2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 look up danh mục</t>
       </text>
     </comment>
-    <comment ref="AL3" authorId="0" shapeId="0">
+    <comment ref="AL2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Danh mục chất liệu</t>
       </text>
     </comment>
-    <comment ref="AM3" authorId="0" shapeId="0">
+    <comment ref="AM2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Yes / No</t>
       </text>
     </comment>
-    <comment ref="AN3" authorId="0" shapeId="0">
+    <comment ref="AN2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Dùng chung danh mục lớp tráng đã có bên thông số mắt</t>
       </text>
     </comment>
-    <comment ref="AO3" authorId="0" shapeId="0">
+    <comment ref="AO2" authorId="0" shapeId="0">
       <text>
         <t>Trung Đỗ Kiên:
 Lookup danh mục mã màu. Và cho chọn nhiều giá trị
 Có dùng chung danh mục với các trường mã màu đã có ko ???</t>
       </text>
     </comment>
-    <comment ref="BG3" authorId="0" shapeId="0">
+    <comment ref="BG2" authorId="0" shapeId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1076,7 +1076,7 @@
     Abbe</t>
       </text>
     </comment>
-    <comment ref="BI3" authorId="0" shapeId="0">
+    <comment ref="BI2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1084,7 +1084,7 @@
     Polarization Efficiency </t>
       </text>
     </comment>
-    <comment ref="BK3" authorId="0" shapeId="0">
+    <comment ref="BK2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1093,7 +1093,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="BR3" authorId="0" shapeId="0">
+    <comment ref="BR2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1286,7 +1286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CE3"/>
+  <dimension ref="A1:CF2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.88" customWidth="1" style="83" min="1" max="1"/>
@@ -1360,607 +1360,552 @@
     <col width="23" customWidth="1" style="92" min="81" max="81"/>
     <col width="15" customWidth="1" style="92" min="82" max="82"/>
     <col width="15" customWidth="1" style="92" min="83" max="83"/>
+    <col width="40" customWidth="1" style="92" min="84" max="84"/>
   </cols>
   <sheetData>
     <row r="1" ht="54" customHeight="1" s="92">
-      <c r="Q1" s="93" t="n"/>
-      <c r="R1" s="93" t="n"/>
-      <c r="S1" s="93" t="n"/>
-      <c r="T1" s="93" t="n"/>
-      <c r="U1" s="93" t="n"/>
-      <c r="V1" s="93" t="n"/>
-      <c r="W1" s="94" t="inlineStr">
-        <is>
-          <t>My thêm cột này (tư vấn nếu phụ kiện có giá riêng, mã riêng mà vẫn bán kèm thì nên qly ntn?</t>
-        </is>
-      </c>
-      <c r="X1" s="93" t="n"/>
-      <c r="Y1" s="93" t="n"/>
-      <c r="Z1" s="93" t="n"/>
-      <c r="AA1" s="95" t="inlineStr">
-        <is>
-          <t>My thêm cột này</t>
-        </is>
-      </c>
-      <c r="AB1" s="93" t="n"/>
-      <c r="AC1" s="93" t="n"/>
-      <c r="AD1" s="95" t="inlineStr">
-        <is>
-          <t>My thêm cột này</t>
-        </is>
-      </c>
-      <c r="AE1" s="93" t="n"/>
-      <c r="AF1" s="93" t="n"/>
-      <c r="AG1" s="93" t="n"/>
-      <c r="AH1" s="93" t="n"/>
-      <c r="AI1" s="93" t="n"/>
-      <c r="AJ1" s="93" t="n"/>
-      <c r="AK1" s="93" t="n"/>
-      <c r="AL1" s="93" t="n"/>
-      <c r="AM1" s="93" t="n"/>
-      <c r="AN1" s="93" t="n"/>
-      <c r="AO1" s="93" t="n"/>
-      <c r="AP1" s="93" t="n"/>
-      <c r="AQ1" s="93" t="n"/>
-      <c r="AR1" s="93" t="n"/>
-      <c r="AS1" s="93" t="n"/>
-      <c r="AT1" s="93" t="n"/>
-      <c r="AU1" s="93" t="n"/>
-      <c r="AV1" s="93" t="n"/>
-      <c r="AW1" s="93" t="n"/>
-      <c r="AX1" s="93" t="n"/>
-      <c r="AY1" s="93" t="n"/>
-      <c r="AZ1" s="93" t="n"/>
-      <c r="BA1" s="93" t="n"/>
-      <c r="BB1" s="93" t="n"/>
-      <c r="BH1" s="91" t="inlineStr">
-        <is>
-          <t>bỏ đi</t>
-        </is>
-      </c>
-      <c r="BI1" s="91" t="inlineStr">
-        <is>
-          <t>bỏ đi</t>
-        </is>
-      </c>
-      <c r="BJ1" s="91" t="inlineStr">
-        <is>
-          <t>bỏ đi</t>
+      <c r="C1" s="97" t="n"/>
+      <c r="D1" s="97" t="n"/>
+      <c r="G1" s="98" t="n"/>
+      <c r="H1" s="99" t="n"/>
+      <c r="I1" s="97" t="n"/>
+      <c r="J1" s="97" t="n"/>
+      <c r="N1" s="97" t="n"/>
+      <c r="R1" s="97" t="n"/>
+      <c r="S1" s="97" t="n"/>
+      <c r="T1" s="100" t="n"/>
+      <c r="U1" s="100" t="n"/>
+      <c r="V1" s="101" t="n"/>
+      <c r="W1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="X1" s="98" t="n"/>
+      <c r="Y1" s="98" t="n"/>
+      <c r="Z1" s="98" t="n"/>
+      <c r="AA1" s="103" t="n"/>
+      <c r="AB1" s="98" t="n"/>
+      <c r="AC1" s="98" t="n"/>
+      <c r="AD1" s="103" t="n"/>
+      <c r="AE1" s="98" t="n"/>
+      <c r="AF1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="AG1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="AH1" s="98" t="n"/>
+      <c r="AI1" s="98" t="n"/>
+      <c r="AJ1" s="98" t="n"/>
+      <c r="AK1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="AL1" s="98" t="n"/>
+      <c r="AM1" s="98" t="n"/>
+      <c r="AN1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="AO1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền</t>
+        </is>
+      </c>
+      <c r="AP1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền</t>
+        </is>
+      </c>
+      <c r="AQ1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền</t>
+        </is>
+      </c>
+      <c r="AR1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền cả só thập phân</t>
+        </is>
+      </c>
+      <c r="AS1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền cả só thập phân</t>
+        </is>
+      </c>
+      <c r="AT1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền cả só thập phân</t>
+        </is>
+      </c>
+      <c r="AU1" s="98" t="inlineStr">
+        <is>
+          <t>cho phép tự điền cả só thập phân</t>
+        </is>
+      </c>
+      <c r="BH1" s="104" t="n"/>
+      <c r="BI1" s="104" t="n"/>
+      <c r="BJ1" s="104" t="n"/>
+      <c r="BM1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="BN1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="BO1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="BS1" s="102" t="inlineStr">
+        <is>
+          <t>được phép ngăn cách bởi dấu phẩy</t>
+        </is>
+      </c>
+      <c r="BY1" s="96" t="inlineStr">
+        <is>
+          <t>ghi màu phủ gương</t>
+        </is>
+      </c>
+      <c r="CF1" s="101" t="inlineStr">
+        <is>
+          <t>1 ảnh/sản phẩm: URL http(s) hoặc đường dẫn file trên máy chủ (nạp vào ảnh chính)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="33.75" customFormat="1" customHeight="1" s="96">
-      <c r="C2" s="97" t="n"/>
-      <c r="D2" s="97" t="n"/>
-      <c r="G2" s="98" t="n"/>
-      <c r="H2" s="99" t="n"/>
-      <c r="I2" s="97" t="n"/>
-      <c r="J2" s="97" t="n"/>
-      <c r="N2" s="97" t="n"/>
-      <c r="R2" s="97" t="n"/>
-      <c r="S2" s="97" t="n"/>
-      <c r="T2" s="100" t="n"/>
-      <c r="U2" s="100" t="n"/>
-      <c r="V2" s="101" t="n"/>
-      <c r="W2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="X2" s="98" t="n"/>
-      <c r="Y2" s="98" t="n"/>
-      <c r="Z2" s="98" t="n"/>
-      <c r="AA2" s="103" t="n"/>
-      <c r="AB2" s="98" t="n"/>
-      <c r="AC2" s="98" t="n"/>
-      <c r="AD2" s="103" t="n"/>
-      <c r="AE2" s="98" t="n"/>
-      <c r="AF2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="AG2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="AH2" s="98" t="n"/>
-      <c r="AI2" s="98" t="n"/>
-      <c r="AJ2" s="98" t="n"/>
-      <c r="AK2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="AL2" s="98" t="n"/>
-      <c r="AM2" s="98" t="n"/>
-      <c r="AN2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="AO2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền</t>
-        </is>
-      </c>
-      <c r="AP2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền</t>
-        </is>
-      </c>
-      <c r="AQ2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền</t>
-        </is>
-      </c>
-      <c r="AR2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền cả só thập phân</t>
-        </is>
-      </c>
-      <c r="AS2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền cả só thập phân</t>
-        </is>
-      </c>
-      <c r="AT2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền cả só thập phân</t>
-        </is>
-      </c>
-      <c r="AU2" s="98" t="inlineStr">
-        <is>
-          <t>cho phép tự điền cả só thập phân</t>
-        </is>
-      </c>
-      <c r="BH2" s="104" t="n"/>
-      <c r="BI2" s="104" t="n"/>
-      <c r="BJ2" s="104" t="n"/>
-      <c r="BM2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="BN2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="BO2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="BS2" s="102" t="inlineStr">
-        <is>
-          <t>được phép ngăn cách bởi dấu phẩy</t>
-        </is>
-      </c>
-      <c r="BY2" s="96" t="inlineStr">
-        <is>
-          <t>ghi màu phủ gương</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="64.90000000000001" customFormat="1" customHeight="1" s="105">
-      <c r="A3" s="106" t="inlineStr">
+      <c r="A2" s="106" t="inlineStr">
         <is>
           <t>Mã số hàng tự sinh</t>
         </is>
       </c>
-      <c r="B3" s="106" t="inlineStr">
+      <c r="B2" s="106" t="inlineStr">
         <is>
           <t>Mã hàng tự đinh nghĩa</t>
         </is>
       </c>
-      <c r="C3" s="107" t="inlineStr">
+      <c r="C2" s="107" t="inlineStr">
         <is>
           <t>Loại hàng</t>
         </is>
       </c>
-      <c r="D3" s="107" t="inlineStr">
+      <c r="D2" s="107" t="inlineStr">
         <is>
           <t>Mã nhóm hàng</t>
         </is>
       </c>
-      <c r="E3" s="108" t="inlineStr">
+      <c r="E2" s="108" t="inlineStr">
         <is>
           <t>Xuất xứ</t>
         </is>
       </c>
-      <c r="F3" s="108" t="inlineStr">
+      <c r="F2" s="108" t="inlineStr">
         <is>
           <t>Ma NCC</t>
         </is>
       </c>
-      <c r="G3" s="109" t="inlineStr">
+      <c r="G2" s="109" t="inlineStr">
         <is>
           <t>Tên nguồn cung cấp</t>
         </is>
       </c>
-      <c r="H3" s="110" t="inlineStr">
+      <c r="H2" s="110" t="inlineStr">
         <is>
           <t>Thương hiệu</t>
         </is>
       </c>
-      <c r="I3" s="107" t="inlineStr">
+      <c r="I2" s="107" t="inlineStr">
         <is>
           <t>Tên đầy đủ</t>
         </is>
       </c>
-      <c r="J3" s="107" t="inlineStr">
+      <c r="J2" s="107" t="inlineStr">
         <is>
           <t>Tên rút gọn</t>
         </is>
       </c>
-      <c r="K3" s="108" t="inlineStr">
+      <c r="K2" s="108" t="inlineStr">
         <is>
           <t>Tên viết hóa đơn</t>
         </is>
       </c>
-      <c r="L3" s="108" t="inlineStr">
+      <c r="L2" s="108" t="inlineStr">
         <is>
           <t>Mã theo NSX (REF)</t>
         </is>
       </c>
-      <c r="M3" s="108" t="inlineStr">
+      <c r="M2" s="108" t="inlineStr">
         <is>
           <t>Mã vạch</t>
         </is>
       </c>
-      <c r="N3" s="111" t="inlineStr">
+      <c r="N2" s="111" t="inlineStr">
         <is>
           <t>Hình thức quản lý (01)</t>
         </is>
       </c>
-      <c r="O3" s="106" t="inlineStr">
+      <c r="O2" s="106" t="inlineStr">
         <is>
           <t>Mã đơn vị tối thiểu</t>
         </is>
       </c>
-      <c r="P3" s="112" t="inlineStr">
+      <c r="P2" s="112" t="inlineStr">
         <is>
           <t>Giá nhập chỉ định chưa thuế</t>
         </is>
       </c>
-      <c r="Q3" s="106" t="inlineStr">
+      <c r="Q2" s="106" t="inlineStr">
         <is>
           <t>Giá bán cơ sở có thuế</t>
         </is>
       </c>
-      <c r="R3" s="111" t="inlineStr">
+      <c r="R2" s="111" t="inlineStr">
         <is>
           <t>Giá bán lẻ có thuế</t>
         </is>
       </c>
-      <c r="S3" s="111" t="inlineStr">
+      <c r="S2" s="111" t="inlineStr">
         <is>
           <t>Giá bán buôn có thuế</t>
         </is>
       </c>
-      <c r="T3" s="111" t="inlineStr">
+      <c r="T2" s="111" t="inlineStr">
         <is>
           <t>Thuế suất mua vào</t>
         </is>
       </c>
-      <c r="U3" s="111" t="inlineStr">
+      <c r="U2" s="111" t="inlineStr">
         <is>
           <t>Mã thuế bán ra</t>
         </is>
       </c>
-      <c r="V3" s="113" t="inlineStr">
+      <c r="V2" s="113" t="inlineStr">
         <is>
           <t>Kiểu in nhãn</t>
         </is>
       </c>
-      <c r="W3" s="114" t="inlineStr">
+      <c r="W2" s="114" t="inlineStr">
         <is>
           <t>Phụ kiện</t>
         </is>
       </c>
-      <c r="X3" s="115" t="inlineStr">
+      <c r="X2" s="115" t="inlineStr">
         <is>
           <t>Mã model</t>
         </is>
       </c>
-      <c r="Y3" s="115" t="inlineStr">
+      <c r="Y2" s="115" t="inlineStr">
         <is>
           <t>Mã màu</t>
         </is>
       </c>
-      <c r="Z3" s="115" t="inlineStr">
+      <c r="Z2" s="115" t="inlineStr">
         <is>
           <t>Loại gọng</t>
         </is>
       </c>
-      <c r="AA3" s="116" t="inlineStr">
+      <c r="AA2" s="116" t="inlineStr">
         <is>
           <t>Cấu trúc vành</t>
         </is>
       </c>
-      <c r="AB3" s="115" t="inlineStr">
+      <c r="AB2" s="115" t="inlineStr">
         <is>
           <t>Giới tính</t>
         </is>
       </c>
-      <c r="AC3" s="115" t="inlineStr">
+      <c r="AC2" s="115" t="inlineStr">
         <is>
           <t>Dáng mắt</t>
         </is>
       </c>
-      <c r="AD3" s="116" t="inlineStr">
+      <c r="AD2" s="116" t="inlineStr">
         <is>
           <t>Loại ve</t>
         </is>
       </c>
-      <c r="AE3" s="115" t="inlineStr">
+      <c r="AE2" s="115" t="inlineStr">
         <is>
           <t>Loại chuôi càng</t>
         </is>
       </c>
-      <c r="AF3" s="115" t="inlineStr">
+      <c r="AF2" s="115" t="inlineStr">
         <is>
           <t>Chất liệu mặt trước</t>
         </is>
       </c>
-      <c r="AG3" s="115" t="inlineStr">
+      <c r="AG2" s="115" t="inlineStr">
         <is>
           <t>Chất liệu càng</t>
         </is>
       </c>
-      <c r="AH3" s="115" t="inlineStr">
+      <c r="AH2" s="115" t="inlineStr">
         <is>
           <t>Trọng lượng (với gọng kính bằng vàng)</t>
         </is>
       </c>
-      <c r="AI3" s="115" t="inlineStr">
+      <c r="AI2" s="115" t="inlineStr">
         <is>
           <t>Số lượng đá quý (kim cương/Saphire) - kèm Carat</t>
         </is>
       </c>
-      <c r="AJ3" s="115" t="inlineStr">
+      <c r="AJ2" s="115" t="inlineStr">
         <is>
           <t>Chất liệu ve</t>
         </is>
       </c>
-      <c r="AK3" s="115" t="inlineStr">
+      <c r="AK2" s="115" t="inlineStr">
         <is>
           <t>Chất liệu chuôi càng</t>
         </is>
       </c>
-      <c r="AL3" s="115" t="inlineStr">
+      <c r="AL2" s="115" t="inlineStr">
         <is>
           <t>Chất liệu mắt</t>
         </is>
       </c>
-      <c r="AM3" s="115" t="inlineStr">
+      <c r="AM2" s="115" t="inlineStr">
         <is>
           <t>Mạ mắt polarized</t>
         </is>
       </c>
-      <c r="AN3" s="115" t="inlineStr">
+      <c r="AN2" s="115" t="inlineStr">
         <is>
           <t>Lớp tráng mắt</t>
         </is>
       </c>
-      <c r="AO3" s="115" t="inlineStr">
+      <c r="AO2" s="115" t="inlineStr">
         <is>
           <t>Màu sắc mặt trước</t>
         </is>
       </c>
-      <c r="AP3" s="115" t="inlineStr">
+      <c r="AP2" s="115" t="inlineStr">
         <is>
           <t>Màu sắc càng kính</t>
         </is>
       </c>
-      <c r="AQ3" s="115" t="inlineStr">
+      <c r="AQ2" s="115" t="inlineStr">
         <is>
           <t>Màu sắc mắt kính</t>
         </is>
       </c>
-      <c r="AR3" s="117" t="inlineStr">
+      <c r="AR2" s="117" t="inlineStr">
         <is>
           <t>Ngang mắt</t>
         </is>
       </c>
-      <c r="AS3" s="115" t="inlineStr">
+      <c r="AS2" s="115" t="inlineStr">
         <is>
           <t xml:space="preserve">Cao mắt </t>
         </is>
       </c>
-      <c r="AT3" s="115" t="inlineStr">
+      <c r="AT2" s="115" t="inlineStr">
         <is>
           <t>Dài cầu</t>
         </is>
       </c>
-      <c r="AU3" s="115" t="inlineStr">
+      <c r="AU2" s="115" t="inlineStr">
         <is>
           <t>Dài càng</t>
         </is>
       </c>
-      <c r="AV3" s="118" t="inlineStr">
+      <c r="AV2" s="123" t="inlineStr">
         <is>
           <t>Loai tròng</t>
         </is>
       </c>
-      <c r="AW3" s="119" t="inlineStr">
+      <c r="AW2" s="119" t="inlineStr">
         <is>
           <t>Cứng/mềm với loại áp tròng</t>
         </is>
       </c>
-      <c r="AX3" s="119" t="inlineStr">
+      <c r="AX2" s="119" t="inlineStr">
         <is>
           <t>Đặc tính</t>
         </is>
       </c>
-      <c r="AY3" s="118" t="inlineStr">
+      <c r="AY2" s="123" t="inlineStr">
         <is>
           <t>Độ cầu</t>
         </is>
       </c>
-      <c r="AZ3" s="118" t="inlineStr">
+      <c r="AZ2" s="123" t="inlineStr">
         <is>
           <t>Độ trụ</t>
         </is>
       </c>
-      <c r="BA3" s="119" t="inlineStr">
+      <c r="BA2" s="119" t="inlineStr">
         <is>
           <t>Độ cộng thêm</t>
         </is>
       </c>
-      <c r="BB3" s="119" t="inlineStr">
+      <c r="BB2" s="119" t="inlineStr">
         <is>
           <t>Trái/Phải</t>
         </is>
       </c>
-      <c r="BC3" s="118" t="inlineStr">
+      <c r="BC2" s="123" t="inlineStr">
         <is>
           <t>Trục</t>
         </is>
       </c>
-      <c r="BD3" s="118" t="inlineStr">
+      <c r="BD2" s="123" t="inlineStr">
         <is>
           <t>Lăng kính</t>
         </is>
       </c>
-      <c r="BE3" s="118" t="inlineStr">
+      <c r="BE2" s="123" t="inlineStr">
         <is>
           <t>Đáy lăng kính</t>
         </is>
       </c>
-      <c r="BF3" s="119" t="inlineStr">
+      <c r="BF2" s="119" t="inlineStr">
         <is>
           <t>Độ cong kính</t>
         </is>
       </c>
-      <c r="BG3" s="119" t="inlineStr">
+      <c r="BG2" s="119" t="inlineStr">
         <is>
           <t>Chỉ số tán sắc</t>
         </is>
       </c>
-      <c r="BH3" s="120" t="inlineStr">
+      <c r="BH2" s="120" t="inlineStr">
         <is>
           <t>Phân cực</t>
         </is>
       </c>
-      <c r="BI3" s="121" t="inlineStr">
+      <c r="BI2" s="121" t="inlineStr">
         <is>
           <t>Hiêu suất phân cực</t>
         </is>
       </c>
-      <c r="BJ3" s="121" t="inlineStr">
+      <c r="BJ2" s="121" t="inlineStr">
         <is>
           <t>Trục phân cực</t>
         </is>
       </c>
-      <c r="BK3" s="119" t="inlineStr">
+      <c r="BK2" s="119" t="inlineStr">
         <is>
           <t>Hạng mục tròng kính</t>
         </is>
       </c>
-      <c r="BL3" s="118" t="inlineStr">
+      <c r="BL2" s="123" t="inlineStr">
         <is>
           <t>Đường kính</t>
         </is>
       </c>
-      <c r="BM3" s="118" t="inlineStr">
+      <c r="BM2" s="123" t="inlineStr">
         <is>
           <t>Thiết kế</t>
         </is>
       </c>
-      <c r="BN3" s="122" t="inlineStr">
+      <c r="BN2" s="122" t="inlineStr">
         <is>
           <t>Lớp film chức năng</t>
         </is>
       </c>
-      <c r="BO3" s="118" t="inlineStr">
+      <c r="BO2" s="123" t="inlineStr">
         <is>
           <t>Chất liệu</t>
         </is>
       </c>
-      <c r="BP3" s="118" t="inlineStr">
+      <c r="BP2" s="123" t="inlineStr">
         <is>
           <t>Chiết suất</t>
         </is>
       </c>
-      <c r="BQ3" s="118" t="inlineStr">
+      <c r="BQ2" s="123" t="inlineStr">
         <is>
           <t>Chống UV</t>
         </is>
       </c>
-      <c r="BR3" s="119" t="inlineStr">
+      <c r="BR2" s="119" t="inlineStr">
         <is>
           <t>Tỷ lệ ánh sáng truyền qua</t>
         </is>
       </c>
-      <c r="BS3" s="118" t="inlineStr">
+      <c r="BS2" s="123" t="inlineStr">
         <is>
           <t>Lớp phủ</t>
         </is>
       </c>
-      <c r="BT3" s="118" t="inlineStr">
+      <c r="BT2" s="123" t="inlineStr">
         <is>
           <t>Ánh mạ</t>
         </is>
       </c>
-      <c r="BU3" s="118" t="inlineStr">
+      <c r="BU2" s="123" t="inlineStr">
         <is>
           <t>Đổi màu</t>
         </is>
       </c>
-      <c r="BV3" s="118" t="inlineStr">
+      <c r="BV2" s="123" t="inlineStr">
         <is>
           <t>Mạ màu</t>
         </is>
       </c>
-      <c r="BW3" s="118" t="inlineStr">
+      <c r="BW2" s="123" t="inlineStr">
         <is>
           <t>Độ đậm màu</t>
         </is>
       </c>
-      <c r="BX3" s="118" t="inlineStr">
+      <c r="BX2" s="123" t="inlineStr">
         <is>
           <t>Corridor</t>
         </is>
       </c>
-      <c r="BY3" s="118" t="inlineStr">
+      <c r="BY2" s="123" t="inlineStr">
         <is>
           <t>Phủ gương</t>
         </is>
       </c>
-      <c r="BZ3" s="123" t="inlineStr">
+      <c r="BZ2" s="123" t="inlineStr">
         <is>
           <t>Thông tin bổ sung</t>
         </is>
       </c>
-      <c r="CA3" s="123" t="inlineStr">
+      <c r="CA2" s="123" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="CB3" s="123" t="inlineStr">
+      <c r="CB2" s="123" t="inlineStr">
         <is>
           <t>Công dụng</t>
         </is>
       </c>
-      <c r="CC3" s="123" t="inlineStr">
+      <c r="CC2" s="123" t="inlineStr">
         <is>
           <t>Hướng dẫn sử dụng</t>
         </is>
       </c>
-      <c r="CD3" s="123" t="inlineStr">
+      <c r="CD2" s="123" t="inlineStr">
         <is>
           <t>Cảnh báo</t>
         </is>
       </c>
-      <c r="CE3" s="123" t="inlineStr">
+      <c r="CE2" s="123" t="inlineStr">
         <is>
           <t>Bảo quản</t>
         </is>
       </c>
-    </row>
+      <c r="CF2" s="108" t="inlineStr">
+        <is>
+          <t>Link ảnh sản phẩm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="64.90000000000001" customFormat="1" customHeight="1" s="105"/>
     <row r="1048404" ht="12.8" customHeight="1" s="92"/>
     <row r="1048405" ht="12.8" customHeight="1" s="92"/>
     <row r="1048406" ht="12.8" customHeight="1" s="92"/>

</xml_diff>